<commit_message>
feat(results): update score sheet template to Cybersentinel 2K26 - CIPHER CODING
</commit_message>
<xml_diff>
--- a/public/Cybersentinel_2K26_Score_Sheet_Template.xlsx
+++ b/public/Cybersentinel_2K26_Score_Sheet_Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36BAFCBE-BA0E-498C-B3AA-FE098D21CFE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CAEF42F-7299-416E-B490-C7EA65B53441}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,17 +17,14 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Evaluation Sheet'!$A$5:$E$15</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Evaluation Sheet'!$A$1:$E$17</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Evaluation Sheet'!$A$1:$E$16</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
-  <si>
-    <t>Cybersentinel 2K26 - WEBLICA</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>Score Sheet</t>
   </si>
@@ -50,14 +47,14 @@
     <t>TIME</t>
   </si>
   <si>
-    <t>Evaluator's Signature: ____________________________________________</t>
+    <t xml:space="preserve">      Cybersentinel 2K26 - CIPHER CODING</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -86,11 +83,6 @@
     <font>
       <sz val="10"/>
       <color rgb="FF111827"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF4B5563"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -145,7 +137,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -162,15 +154,12 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -557,7 +546,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -568,21 +557,21 @@
   <sheetData>
     <row r="1" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="6" t="s">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="C1" s="7"/>
       <c r="D1" s="7"/>
     </row>
     <row r="2" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="8" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C2" s="7"/>
       <c r="D2" s="7"/>
     </row>
     <row r="3" spans="1:5" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="10" t="s">
-        <v>2</v>
+      <c r="B3" s="9" t="s">
+        <v>1</v>
       </c>
       <c r="C3" s="7"/>
       <c r="D3" s="7"/>
@@ -590,19 +579,19 @@
     <row r="4" spans="1:5" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="5" spans="1:5" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="C5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="D5" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="E5" s="1" t="s">
         <v>6</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="30.95" customHeight="1" x14ac:dyDescent="0.25">
@@ -675,21 +664,11 @@
       <c r="D15" s="4"/>
       <c r="E15" s="4"/>
     </row>
-    <row r="17" spans="1:5" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="B17" s="7"/>
-      <c r="C17" s="7"/>
-      <c r="D17" s="7"/>
-      <c r="E17" s="7"/>
-    </row>
   </sheetData>
   <autoFilter ref="A5:E15" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
-  <mergeCells count="4">
+  <mergeCells count="3">
     <mergeCell ref="B1:D1"/>
     <mergeCell ref="B2:D2"/>
-    <mergeCell ref="A17:E17"/>
     <mergeCell ref="B3:D3"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.35" bottom="0.35" header="0.5" footer="0.5"/>

</xml_diff>